<commit_message>
feat(preseg): T7 块流→ChunkSpec 适配器 + s3 分支 + entity_type 继承(D7)
adapter:章/节标题块更新上下文不成块(与条款树一致);norm=章/节/条上下文拼接(label 内嵌
优先);同 norm 多块 seq 递增防撞 id;超预算复用 _split_oversize(句末语义切/无边界硬切标
oversize);推导失败落 preseg/{block_seq}+chunk_type=preseg_raw;零页码(D2);**搬运保真:
源块文本原样入 chunk,不加前缀不改写**。s3 分支:preseg 文档直接消费 raw 块流(clause_label
全保真不经 IR);preseg 案例暂走 case_chunker,T9 换直装。D7 载体补差:manifest/dv 增
entity_types 列(迁移 0014,T3/T4 遗漏),ChunkSpec/_to_row/chunks.entity_type 写入路径打通
(corpus_rows 投影既有,零改)。12 纯函数测 + s3 真栈集成测;chunking 波及面 89 passed 回归绿。
(SPEC-PRESEG §3.3/§4-S3 / TASKS T7)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/tests/fixtures/preseg_batch/manifest.xlsx
+++ b/pipeline/tests/fixtures/preseg_batch/manifest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,15 +494,20 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>entity_types</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>file_no</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>source_created_by</t>
         </is>
@@ -582,11 +587,16 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>证券公司;证券从业人员</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>招揽;展业</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
         <is>
           <t>kb_admin</t>
         </is>
@@ -664,17 +674,18 @@
           <t>公司级</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>合规</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>ZD-2024-005</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>kb_admin</t>
         </is>

</xml_diff>

<commit_message>
feat(preseg/reader): CP-010 P1 接收契约扩展(源锚 + 版本/效力列)
扩展 intake 接收契约以承载真 schema 的结构数据(沿用 Codex 四轮"坏类型整文件拒收"严校验):
- blocks JSONL +source_code(LAW_CONTENT.CODE,精确桥接锚)、+clause_path_norm
  (源 PATH_CODE 算好的权威 norm,缺→adapter 回落 derive)、+is_catalog(IS_CATALOG==1 目录块)
- violated_regulations +law_code/law_content_code(CASE_PUNISH 的精确条款外键)
- manifest PRESEG_EXTRA_COLUMNS +source_law_id/invalid_date;fixture manifest 重生成为 21 列

blocks_content_hash canon 纳入三新字段:clause_path_norm 进 chunk_id、source_code 决定桥接、
is_catalog 决定成不成块,不纳入则"仅改结构元数据"的变化件被误判 DUPLICATE 漏更新
(preseg 未上真环境,改 canon 无存量哈希冲突)。

契约破坏性变更(SPEC §7 Ask-first)已由用户"捕获结构红利"决策授权,转换脚本(P5)按新契约产出。
test_preseg_reader +12 例(新字段解析/严校验/指纹敏感性)。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/tests/fixtures/preseg_batch/manifest.xlsx
+++ b/pipeline/tests/fixtures/preseg_batch/manifest.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="manifest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,16 @@
           <t>source_created_by</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_law_id</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>invalid_date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -564,7 +574,6 @@
           <t>2024-03-01</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>KB-EXT-0001</t>
@@ -595,10 +604,14 @@
           <t>招揽;展业</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>kb_admin</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>KB-EXT-0000-PRE</t>
         </is>
       </c>
     </row>
@@ -653,7 +666,6 @@
           <t>2024-05-01</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>KB-INT-0001</t>
@@ -674,7 +686,6 @@
           <t>公司级</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>合规</t>
@@ -688,6 +699,11 @@
       <c r="S3" t="inlineStr">
         <is>
           <t>kb_admin</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
         </is>
       </c>
     </row>

</xml_diff>